<commit_message>
Let clients skip any question or section
The AI moves on without asking why or guessing an answer, and records
'不清楚' (don't know) and '（跳过）' (skipped) separately so the FDE can
tell why a cell is empty. Template instructions and docs updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fde-pre-visit-intake/template/intake_form.xlsx
+++ b/fde-pre-visit-intake/template/intake_form.xlsx
@@ -632,7 +632,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>4</t>
@@ -640,7 +640,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>不确定、不知道的地方空着，我们上门时再一起确认。</t>
+          <t>任何问题都可以跳过，不需要说明原因：不知道的写“不清楚”，不想回答的写“跳过”或直接空着。我们上门时再一起确认。</t>
         </is>
       </c>
     </row>

</xml_diff>